<commit_message>
Update import template example XLSX files
Add new example templates and refresh existing ones under ImportTemplate. New files added: fungi-example-01.xlsx, animals-example-01.xlsx. Updated binary Excel files: product-example-01.xlsx, expert-example-01.xlsx, ecotourism-example-01.xlsx. These are example import templates (binary .xlsx) for various data types.
</commit_message>
<xml_diff>
--- a/ImportTemplate/ผลิตภัณฑ์/product-example-01.xlsx
+++ b/ImportTemplate/ผลิตภัณฑ์/product-example-01.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\biog\biog\ImportTemplate\ตัวอย่าง\ผลิตภัณฑ์\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\biog\biog\ImportTemplate\ผลิตภัณฑ์\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5008126D-2D67-4867-B7DC-7A97546B2991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BCCF91C-AB7A-4358-9881-299647BD630D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5989159A-E7FB-42B4-9C9A-65CB7C17A329}"/>
   </bookViews>
@@ -37,9 +37,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="74">
   <si>
-    <t>Template Import เนื้อหา ประเภทพืช</t>
-  </si>
-  <si>
     <t>ชื่อเรือง</t>
   </si>
   <si>
@@ -257,6 +254,9 @@
   </si>
   <si>
     <t>product_01_gallery_01.jpg, product_01_gallery_02.jpg</t>
+  </si>
+  <si>
+    <t>Template Import เนื้อหา ผลิตภัณฑ์</t>
   </si>
 </sst>
 </file>
@@ -362,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -379,32 +379,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="7">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -422,6 +416,9 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -557,7 +554,7 @@
     <tableColumn id="18" xr3:uid="{686DDB6E-598B-4F52-B899-2284742E96CC}" name="แหล่งที่พบ"/>
     <tableColumn id="26" xr3:uid="{B860955C-A1E0-483E-B81F-BCC39EFA8534}" name="ข้อมูลการติดต่อ"/>
     <tableColumn id="19" xr3:uid="{F012D379-D3FE-47CF-A848-752A5BA35121}" name="รูปประกอบ (แสดงเป็น Gallery)"/>
-    <tableColumn id="20" xr3:uid="{20D1F43B-4271-4C25-A8BA-9B5959DF5076}" name="คำสำคัญ (Tags)" dataDxfId="0">
+    <tableColumn id="20" xr3:uid="{20D1F43B-4271-4C25-A8BA-9B5959DF5076}" name="คำสำคัญ (Tags)" dataDxfId="1">
       <calculatedColumnFormula array="1">ผลิตภัณฑ์จักสานจากไม้ไผ่</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="21" xr3:uid="{71E71F89-EE0D-4C69-AD0C-36F0DCB00B9C}" name="หมายเหตุ"/>
@@ -595,7 +592,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4D48FDCA-27DA-4B3E-8695-D26F77EBF2A7}" name="Table35" displayName="Table35" ref="H5:I12" totalsRowShown="0">
   <autoFilter ref="H5:I12" xr:uid="{4D48FDCA-27DA-4B3E-8695-D26F77EBF2A7}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{923B0286-770F-4246-AFFD-1EA693646F62}" name="value" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{923B0286-770F-4246-AFFD-1EA693646F62}" name="value" dataDxfId="0"/>
     <tableColumn id="2" xr3:uid="{5078F3B0-C3C6-410C-9026-208DE4DBC7FC}" name="label"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -941,211 +938,211 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+    </row>
+    <row r="2" spans="1:26" ht="17.25" thickBot="1">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8"/>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
-    </row>
-    <row r="2" spans="1:26" ht="50.25" thickBot="1">
-      <c r="A2" s="4" t="s">
+      <c r="B2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="S2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="P2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="Q2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="R2" s="4" t="s">
+      <c r="U2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="W2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="S2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="T2" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="U2" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="W2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="Z2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="Z2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:26" ht="86.25" customHeight="1" thickBot="1">
+      <c r="A3" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="8">
+        <v>80</v>
+      </c>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="T3" s="8"/>
+      <c r="U3" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="V3" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="W3" s="8"/>
+      <c r="X3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z3" s="8" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" ht="86.25" customHeight="1" thickBot="1">
-      <c r="A3" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" s="10">
-        <v>80</v>
-      </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="N3" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="T3" s="10"/>
-      <c r="U3" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="V3" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="W3" s="10"/>
-      <c r="X3" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y3" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="Z3" s="10" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="30.75" thickBot="1">
       <c r="A4" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D4" s="7">
         <v>30</v>
       </c>
       <c r="F4" t="s">
+        <v>59</v>
+      </c>
+      <c r="M4" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="N4" t="s">
         <v>61</v>
       </c>
-      <c r="N4" t="s">
+      <c r="P4" t="s">
         <v>62</v>
       </c>
-      <c r="P4" t="s">
+      <c r="S4" t="s">
         <v>63</v>
       </c>
-      <c r="S4" t="s">
+      <c r="U4" t="s">
         <v>64</v>
       </c>
-      <c r="U4" t="s">
-        <v>65</v>
-      </c>
       <c r="V4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="X4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Y4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="Z4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36" spans="2:2">
@@ -1219,43 +1216,43 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:11">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="12"/>
+      <c r="E4" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="E4" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="9"/>
-      <c r="H4" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="I4" s="9"/>
+      <c r="F4" s="12"/>
+      <c r="H4" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="12"/>
       <c r="K4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="2:11">
       <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
-        <v>17</v>
-      </c>
       <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" t="s">
         <v>16</v>
       </c>
-      <c r="F5" t="s">
-        <v>17</v>
-      </c>
       <c r="H5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" t="s">
         <v>16</v>
       </c>
-      <c r="I5" t="s">
-        <v>17</v>
-      </c>
       <c r="K5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="2:11">
@@ -1263,22 +1260,22 @@
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" t="s">
         <v>21</v>
       </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
       <c r="H6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="K6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="2:11">
@@ -1286,71 +1283,71 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="2:11">
       <c r="E8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="2:11">
       <c r="H9" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="2:11">
       <c r="H10" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="2:11">
       <c r="H11" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="2:11">
       <c r="H12" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>